<commit_message>
Auto commit every 30 seconds [no ci]
</commit_message>
<xml_diff>
--- a/Projects/ai-docx/penjualan_produk_2024.xlsx
+++ b/Projects/ai-docx/penjualan_produk_2024.xlsx
@@ -445,7 +445,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>351</v>
+        <v>814</v>
       </c>
     </row>
     <row r="3">
@@ -460,7 +460,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>148</v>
+        <v>735</v>
       </c>
     </row>
     <row r="4">
@@ -475,7 +475,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>816</v>
+        <v>399</v>
       </c>
     </row>
     <row r="5">
@@ -490,7 +490,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>848</v>
+        <v>412</v>
       </c>
     </row>
     <row r="6">
@@ -505,7 +505,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>418</v>
+        <v>440</v>
       </c>
     </row>
     <row r="7">
@@ -520,7 +520,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>598</v>
+        <v>228</v>
       </c>
     </row>
     <row r="8">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>395</v>
+        <v>870</v>
       </c>
     </row>
     <row r="9">
@@ -550,7 +550,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>230</v>
+        <v>208</v>
       </c>
     </row>
     <row r="10">
@@ -565,7 +565,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>833</v>
+        <v>550</v>
       </c>
     </row>
     <row r="11">
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>243</v>
+        <v>726</v>
       </c>
     </row>
     <row r="12">
@@ -595,7 +595,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>411</v>
+        <v>716</v>
       </c>
     </row>
     <row r="13">
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>869</v>
+        <v>661</v>
       </c>
     </row>
     <row r="14">
@@ -625,7 +625,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>735</v>
+        <v>510</v>
       </c>
     </row>
     <row r="15">
@@ -640,7 +640,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>811</v>
+        <v>309</v>
       </c>
     </row>
     <row r="16">
@@ -655,7 +655,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>659</v>
+        <v>206</v>
       </c>
     </row>
     <row r="17">
@@ -670,7 +670,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>699</v>
+        <v>802</v>
       </c>
     </row>
     <row r="18">
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>937</v>
+        <v>324</v>
       </c>
     </row>
     <row r="19">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>101</v>
+        <v>799</v>
       </c>
     </row>
     <row r="20">
@@ -715,7 +715,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>811</v>
+        <v>752</v>
       </c>
     </row>
     <row r="21">
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>935</v>
+        <v>130</v>
       </c>
     </row>
     <row r="22">
@@ -745,7 +745,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>572</v>
+        <v>762</v>
       </c>
     </row>
     <row r="23">
@@ -760,7 +760,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>684</v>
+        <v>434</v>
       </c>
     </row>
     <row r="24">
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>577</v>
+        <v>923</v>
       </c>
     </row>
     <row r="25">
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>261</v>
+        <v>665</v>
       </c>
     </row>
     <row r="26">
@@ -805,7 +805,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>492</v>
+        <v>728</v>
       </c>
     </row>
     <row r="27">
@@ -820,7 +820,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>330</v>
+        <v>919</v>
       </c>
     </row>
     <row r="28">
@@ -835,7 +835,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>454</v>
+        <v>930</v>
       </c>
     </row>
     <row r="29">
@@ -850,7 +850,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>897</v>
+        <v>785</v>
       </c>
     </row>
     <row r="30">
@@ -865,7 +865,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>642</v>
+        <v>764</v>
       </c>
     </row>
     <row r="31">
@@ -880,7 +880,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>181</v>
+        <v>397</v>
       </c>
     </row>
     <row r="32">
@@ -895,7 +895,7 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>789</v>
+        <v>436</v>
       </c>
     </row>
     <row r="33">
@@ -910,7 +910,7 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>327</v>
+        <v>938</v>
       </c>
     </row>
     <row r="34">
@@ -925,7 +925,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>886</v>
+        <v>760</v>
       </c>
     </row>
     <row r="35">
@@ -940,7 +940,7 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>927</v>
+        <v>404</v>
       </c>
     </row>
     <row r="36">
@@ -955,7 +955,7 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>720</v>
+        <v>237</v>
       </c>
     </row>
     <row r="37">
@@ -970,7 +970,7 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>602</v>
+        <v>936</v>
       </c>
     </row>
   </sheetData>

</xml_diff>